<commit_message>
auto: actualizar indicadores adelantados 2026-09-28
</commit_message>
<xml_diff>
--- a/datos/indicadores_adelantados/energia/indice_consumo_energia_electrica_2017_2026.xlsx
+++ b/datos/indicadores_adelantados/energia/indice_consumo_energia_electrica_2017_2026.xlsx
@@ -4533,25 +4533,25 @@
         <v>33</v>
       </c>
       <c r="C132" s="10">
-        <v>125.145180201377</v>
+        <v>122.88877997023801</v>
       </c>
       <c r="D132" s="10">
-        <v>126.899692551635</v>
+        <v>122.15094187733</v>
       </c>
       <c r="E132" s="10">
-        <v>118.274828201093</v>
+        <v>117.300517005877</v>
       </c>
       <c r="F132" s="10">
-        <v>180.94476445483599</v>
+        <v>183.181873589394</v>
       </c>
       <c r="G132" s="10">
-        <v>116.691000897694</v>
+        <v>112.019864578366</v>
       </c>
       <c r="H132" s="10">
-        <v>160.687613248579</v>
+        <v>158.93205939791699</v>
       </c>
       <c r="I132" s="10">
-        <v>127.89020849115001</v>
+        <v>125.259801752</v>
       </c>
     </row>
     <row r="133" spans="2:9">
@@ -4559,25 +4559,25 @@
         <v>6</v>
       </c>
       <c r="C133" s="12">
-        <v>133.81745310174699</v>
+        <v>133.13831198384199</v>
       </c>
       <c r="D133" s="12">
-        <v>130.315067629449</v>
+        <v>127.271341585988</v>
       </c>
       <c r="E133" s="12">
-        <v>117.55876343064899</v>
+        <v>115.834787463176</v>
       </c>
       <c r="F133" s="12">
         <v>171.086962259134</v>
       </c>
       <c r="G133" s="12">
-        <v>115.76923599584499</v>
+        <v>110.277862718798</v>
       </c>
       <c r="H133" s="12">
-        <v>152.85179416885401</v>
+        <v>149.66492868690699</v>
       </c>
       <c r="I133" s="12">
-        <v>131.275379933279</v>
+        <v>129.39004974020199</v>
       </c>
     </row>
     <row r="134" spans="2:9">
@@ -4585,25 +4585,25 @@
         <v>7</v>
       </c>
       <c r="C134" s="12">
-        <v>130.45201169262</v>
+        <v>129.776778725421</v>
       </c>
       <c r="D134" s="12">
-        <v>130.87266117091599</v>
+        <v>127.81869034118699</v>
       </c>
       <c r="E134" s="12">
-        <v>117.192635509624</v>
+        <v>115.47076275844501</v>
       </c>
       <c r="F134" s="12">
         <v>173.441249375523</v>
       </c>
       <c r="G134" s="12">
-        <v>100.571432663838</v>
+        <v>95.569212828195006</v>
       </c>
       <c r="H134" s="12">
-        <v>153.57623840542101</v>
+        <v>150.55281705313101</v>
       </c>
       <c r="I134" s="12">
-        <v>129.26183797899</v>
+        <v>127.411331799864</v>
       </c>
     </row>
     <row r="135" spans="2:9">
@@ -4611,25 +4611,25 @@
         <v>8</v>
       </c>
       <c r="C135" s="12">
-        <v>128.84501269150601</v>
+        <v>128.221799364887</v>
       </c>
       <c r="D135" s="12">
-        <v>130.74387424263199</v>
+        <v>127.69149669452</v>
       </c>
       <c r="E135" s="12">
-        <v>124.35357664608399</v>
+        <v>122.65883552751799</v>
       </c>
       <c r="F135" s="12">
         <v>168.02622962471301</v>
       </c>
       <c r="G135" s="12">
-        <v>112.84721877291901</v>
+        <v>107.467631901583</v>
       </c>
       <c r="H135" s="12">
-        <v>168.68080390186901</v>
+        <v>165.62477124564001</v>
       </c>
       <c r="I135" s="12">
-        <v>130.91635057244599</v>
+        <v>129.06711750235101</v>
       </c>
     </row>
     <row r="136" spans="2:9">
@@ -4637,25 +4637,25 @@
         <v>9</v>
       </c>
       <c r="C136" s="12">
-        <v>130.06703932590801</v>
+        <v>129.56092972302201</v>
       </c>
       <c r="D136" s="12">
-        <v>135.09732653873701</v>
+        <v>132.03452004017501</v>
       </c>
       <c r="E136" s="12">
-        <v>130.94791723485801</v>
+        <v>129.16564495852299</v>
       </c>
       <c r="F136" s="12">
         <v>191.016110680964</v>
       </c>
       <c r="G136" s="12">
-        <v>131.75569020193799</v>
+        <v>126.486472253092</v>
       </c>
       <c r="H136" s="12">
-        <v>161.671217884187</v>
+        <v>158.12208171700701</v>
       </c>
       <c r="I136" s="12">
-        <v>135.89738379486101</v>
+        <v>134.06453787532701</v>
       </c>
     </row>
     <row r="137" spans="2:9">
@@ -4663,25 +4663,25 @@
         <v>10</v>
       </c>
       <c r="C137" s="12">
-        <v>116.575808699818</v>
+        <v>116.153352096899</v>
       </c>
       <c r="D137" s="12">
-        <v>121.813157685467</v>
+        <v>119.03259659536199</v>
       </c>
       <c r="E137" s="12">
-        <v>119.14422829253201</v>
+        <v>117.603891163109</v>
       </c>
       <c r="F137" s="12">
         <v>187.73390481546099</v>
       </c>
       <c r="G137" s="12">
-        <v>120.60731993097301</v>
+        <v>115.090461712289</v>
       </c>
       <c r="H137" s="12">
-        <v>160.94685180598799</v>
+        <v>157.631959331639</v>
       </c>
       <c r="I137" s="12">
-        <v>123.870834517403</v>
+        <v>122.18709595877699</v>
       </c>
     </row>
     <row r="138" spans="2:9">
@@ -4689,38 +4689,52 @@
         <v>11</v>
       </c>
       <c r="C138" s="12">
-        <v>111.113755696665</v>
+        <v>110.759533101789</v>
       </c>
       <c r="D138" s="12">
-        <v>112.556068042611</v>
+        <v>109.73253555183901</v>
       </c>
       <c r="E138" s="12">
-        <v>100.45184809281</v>
+        <v>98.978303686929806</v>
       </c>
       <c r="F138" s="12">
         <v>194.36412997321901</v>
       </c>
       <c r="G138" s="12">
-        <v>118.59510782065399</v>
+        <v>113.32452378587899</v>
       </c>
       <c r="H138" s="12">
-        <v>166.39877332515599</v>
+        <v>162.77449867730201</v>
       </c>
       <c r="I138" s="12">
-        <v>116.119464149923</v>
+        <v>114.46685207767401</v>
       </c>
     </row>
     <row r="139" spans="2:9">
       <c r="B139" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="C139" s="16"/>
-      <c r="D139" s="16"/>
-      <c r="E139" s="16"/>
-      <c r="F139" s="16"/>
-      <c r="G139" s="16"/>
-      <c r="H139" s="16"/>
-      <c r="I139" s="16"/>
+      <c r="C139" s="16">
+        <v>112.61075479580801</v>
+      </c>
+      <c r="D139" s="16">
+        <v>111.47541233224</v>
+      </c>
+      <c r="E139" s="16">
+        <v>121.39139348344099</v>
+      </c>
+      <c r="F139" s="16">
+        <v>196.60452839674201</v>
+      </c>
+      <c r="G139" s="16">
+        <v>115.922886848723</v>
+      </c>
+      <c r="H139" s="16">
+        <v>168.15335907379099</v>
+      </c>
+      <c r="I139" s="16">
+        <v>120.23162730980199</v>
+      </c>
     </row>
     <row r="140" spans="2:9" ht="14.25" customHeight="1">
       <c r="B140" s="29" t="s">
@@ -7891,25 +7905,25 @@
         <v>33</v>
       </c>
       <c r="C118" s="10">
-        <v>3.6360074606287802</v>
+        <v>3.1992428821396399</v>
       </c>
       <c r="D118" s="10">
-        <v>1.8616319233407901</v>
+        <v>-0.341613721558645</v>
       </c>
       <c r="E118" s="10">
-        <v>-8.3048776292568203</v>
+        <v>-9.7537102968022502</v>
       </c>
       <c r="F118" s="10">
-        <v>16.2847842921989</v>
+        <v>16.067307000241101</v>
       </c>
       <c r="G118" s="10">
-        <v>0.71257925509588904</v>
+        <v>-4.0999840497543003</v>
       </c>
       <c r="H118" s="10">
-        <v>5.49063354222044</v>
+        <v>3.2118276840339899</v>
       </c>
       <c r="I118" s="10">
-        <v>1.87263882516264</v>
+        <v>0.45838146946684299</v>
       </c>
       <c r="J118" s="1"/>
       <c r="K118" s="1"/>
@@ -7919,25 +7933,25 @@
         <v>6</v>
       </c>
       <c r="C119" s="12">
-        <v>7.3000843336288801</v>
+        <v>6.7555223386386798</v>
       </c>
       <c r="D119" s="12">
-        <v>0.32419331379016603</v>
+        <v>-2.0190457723200401</v>
       </c>
       <c r="E119" s="12">
-        <v>-8.9783131613286002</v>
+        <v>-10.313128159798</v>
       </c>
       <c r="F119" s="12">
         <v>-11.3296548989108</v>
       </c>
       <c r="G119" s="12">
-        <v>5.1591213604943702</v>
+        <v>0.17102600070926199</v>
       </c>
       <c r="H119" s="12">
-        <v>-10.837545071435599</v>
+        <v>-12.696527175261201</v>
       </c>
       <c r="I119" s="12">
-        <v>0.44593016463887503</v>
+        <v>-0.99663846481280505</v>
       </c>
       <c r="J119" s="1"/>
       <c r="K119" s="1"/>
@@ -7947,25 +7961,25 @@
         <v>7</v>
       </c>
       <c r="C120" s="12">
-        <v>-2.5149495309616499</v>
+        <v>-2.5248429308832301</v>
       </c>
       <c r="D120" s="12">
-        <v>0.42788109741207497</v>
+        <v>0.43006441857098598</v>
       </c>
       <c r="E120" s="12">
-        <v>-0.31144247382378598</v>
+        <v>-0.31426198701000102</v>
       </c>
       <c r="F120" s="12">
         <v>1.37607628617773</v>
       </c>
       <c r="G120" s="12">
-        <v>-13.127670059558801</v>
+        <v>-13.337808267203201</v>
       </c>
       <c r="H120" s="12">
-        <v>0.47395206612104201</v>
+        <v>0.59325078628282801</v>
       </c>
       <c r="I120" s="12">
-        <v>-1.5338306050327</v>
+        <v>-1.5292659244748299</v>
       </c>
       <c r="J120" s="1"/>
       <c r="K120" s="1"/>
@@ -7975,25 +7989,25 @@
         <v>8</v>
       </c>
       <c r="C121" s="12">
-        <v>-1.23186985027123</v>
+        <v>-1.19819537501703</v>
       </c>
       <c r="D121" s="12">
-        <v>-9.8406288319763405E-2</v>
+        <v>-9.9510991959073106E-2</v>
       </c>
       <c r="E121" s="12">
-        <v>6.11040199353834</v>
+        <v>6.2250154042107004</v>
       </c>
       <c r="F121" s="12">
         <v>-3.12210605626229</v>
       </c>
       <c r="G121" s="12">
-        <v>12.2060368276878</v>
+        <v>12.450054490642</v>
       </c>
       <c r="H121" s="12">
-        <v>9.8352229832417297</v>
+        <v>10.011074178167</v>
       </c>
       <c r="I121" s="12">
-        <v>1.27996988076684</v>
+        <v>1.2995592143152199</v>
       </c>
       <c r="J121" s="1"/>
       <c r="K121" s="1"/>
@@ -8003,25 +8017,25 @@
         <v>9</v>
       </c>
       <c r="C122" s="12">
-        <v>0.94844698205578404</v>
+        <v>1.04438587258016</v>
       </c>
       <c r="D122" s="12">
-        <v>3.3297562285986801</v>
+        <v>3.4011844626155501</v>
       </c>
       <c r="E122" s="12">
-        <v>5.3028957965092403</v>
+        <v>5.3048028729613099</v>
       </c>
       <c r="F122" s="12">
         <v>13.682316807083801</v>
       </c>
       <c r="G122" s="12">
-        <v>16.755815193875701</v>
+        <v>17.6972731370189</v>
       </c>
       <c r="H122" s="12">
-        <v>-4.1555327313707</v>
+        <v>-4.5299320096910396</v>
       </c>
       <c r="I122" s="12">
-        <v>3.80474493876015</v>
+        <v>3.8719547392734399</v>
       </c>
       <c r="J122" s="1"/>
       <c r="K122" s="1"/>
@@ -8031,25 +8045,25 @@
         <v>10</v>
       </c>
       <c r="C123" s="12">
-        <v>-10.372520737006401</v>
+        <v>-10.3484728419173</v>
       </c>
       <c r="D123" s="12">
-        <v>-9.8330360737828997</v>
+        <v>-9.8473667650375099</v>
       </c>
       <c r="E123" s="12">
-        <v>-9.0140333588935899</v>
+        <v>-8.9511059996845095</v>
       </c>
       <c r="F123" s="12">
         <v>-1.7182874542895901</v>
       </c>
       <c r="G123" s="12">
-        <v>-8.4613956739772007</v>
+        <v>-9.0096674670474002</v>
       </c>
       <c r="H123" s="12">
-        <v>-0.44804887825982098</v>
+        <v>-0.30996454135048301</v>
       </c>
       <c r="I123" s="12">
-        <v>-8.8497283329695406</v>
+        <v>-8.8594956614067701</v>
       </c>
       <c r="J123" s="1"/>
       <c r="K123" s="1"/>
@@ -8059,25 +8073,25 @@
         <v>11</v>
       </c>
       <c r="C124" s="12">
-        <v>-4.6854086315777401</v>
+        <v>-4.6437049794399696</v>
       </c>
       <c r="D124" s="12">
-        <v>-7.5994168600068397</v>
+        <v>-7.81303719277635</v>
       </c>
       <c r="E124" s="12">
-        <v>-15.6888675747067</v>
+        <v>-15.837560553457299</v>
       </c>
       <c r="F124" s="12">
         <v>3.5317142975718201</v>
       </c>
       <c r="G124" s="12">
-        <v>-1.66839965556889</v>
+        <v>-1.53439120856474</v>
       </c>
       <c r="H124" s="12">
-        <v>3.3874048842783302</v>
+        <v>3.26237101122608</v>
       </c>
       <c r="I124" s="12">
-        <v>-6.2576234330533502</v>
+        <v>-6.3183790567443499</v>
       </c>
       <c r="J124" s="1"/>
       <c r="K124" s="1"/>
@@ -8086,13 +8100,27 @@
       <c r="B125" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="C125" s="16"/>
-      <c r="D125" s="16"/>
-      <c r="E125" s="16"/>
-      <c r="F125" s="16"/>
-      <c r="G125" s="16"/>
-      <c r="H125" s="16"/>
-      <c r="I125" s="16"/>
+      <c r="C125" s="16">
+        <v>1.67138813443486</v>
+      </c>
+      <c r="D125" s="16">
+        <v>1.58829536894929</v>
+      </c>
+      <c r="E125" s="16">
+        <v>22.644447279481099</v>
+      </c>
+      <c r="F125" s="16">
+        <v>1.1526810136374599</v>
+      </c>
+      <c r="G125" s="16">
+        <v>2.2928515170759698</v>
+      </c>
+      <c r="H125" s="16">
+        <v>3.3044859238994699</v>
+      </c>
+      <c r="I125" s="16">
+        <v>5.0361961803725697</v>
+      </c>
       <c r="J125" s="1"/>
       <c r="K125" s="1"/>
     </row>
@@ -11227,25 +11255,25 @@
         <v>37</v>
       </c>
       <c r="C118" s="10">
-        <v>3.6360074606287802</v>
+        <v>3.1992428821396399</v>
       </c>
       <c r="D118" s="10">
-        <v>1.8616319233407901</v>
+        <v>-0.341613721558645</v>
       </c>
       <c r="E118" s="10">
-        <v>-8.3048776292568203</v>
+        <v>-9.7537102968022502</v>
       </c>
       <c r="F118" s="10">
-        <v>16.2847842921989</v>
+        <v>16.067307000241101</v>
       </c>
       <c r="G118" s="10">
-        <v>0.71257925509588904</v>
+        <v>-4.0999840497543003</v>
       </c>
       <c r="H118" s="10">
-        <v>5.49063354222044</v>
+        <v>3.2118276840339899</v>
       </c>
       <c r="I118" s="10">
-        <v>1.87263882516264</v>
+        <v>0.45838146946684299</v>
       </c>
       <c r="K118" s="1"/>
     </row>
@@ -11254,25 +11282,25 @@
         <v>6</v>
       </c>
       <c r="C119" s="12">
-        <v>3.72865534857034</v>
+        <v>3.20221882389218</v>
       </c>
       <c r="D119" s="12">
-        <v>2.7518191852456502</v>
+        <v>0.35187884253371499</v>
       </c>
       <c r="E119" s="12">
-        <v>-2.5515743658463301</v>
+        <v>-3.98063621507624</v>
       </c>
       <c r="F119" s="12">
         <v>13.293318580951601</v>
       </c>
       <c r="G119" s="12">
-        <v>6.0160708382844801</v>
+        <v>0.987327119532178</v>
       </c>
       <c r="H119" s="12">
-        <v>-5.3865980203131096</v>
+        <v>-7.3592290027508902</v>
       </c>
       <c r="I119" s="12">
-        <v>2.9091867005634802</v>
+        <v>1.43124165915374</v>
       </c>
       <c r="K119" s="1"/>
     </row>
@@ -11281,25 +11309,25 @@
         <v>7</v>
       </c>
       <c r="C120" s="12">
-        <v>-1.0685583386863899</v>
+        <v>-1.5806376085685101</v>
       </c>
       <c r="D120" s="12">
-        <v>-0.39487759249986498</v>
+        <v>-2.7192067197782999</v>
       </c>
       <c r="E120" s="12">
-        <v>-6.3271279247704504</v>
+        <v>-7.7034325470668499</v>
       </c>
       <c r="F120" s="12">
         <v>14.561465258757099</v>
       </c>
       <c r="G120" s="12">
-        <v>-6.4227956839202101</v>
+        <v>-11.077136734808199</v>
       </c>
       <c r="H120" s="12">
-        <v>4.76202309158404</v>
+        <v>2.69959637236752</v>
       </c>
       <c r="I120" s="12">
-        <v>-0.83320959179789</v>
+        <v>-2.2528765351399498</v>
       </c>
       <c r="K120" s="1"/>
     </row>
@@ -11308,25 +11336,25 @@
         <v>8</v>
       </c>
       <c r="C121" s="12">
-        <v>1.45931237591159</v>
+        <v>0.96856155629183605</v>
       </c>
       <c r="D121" s="12">
-        <v>0.76245692349070604</v>
+        <v>-1.58996733338195</v>
       </c>
       <c r="E121" s="12">
-        <v>3.3733094604205101</v>
+        <v>1.96449595597716</v>
       </c>
       <c r="F121" s="12">
         <v>19.799265689296799</v>
       </c>
       <c r="G121" s="12">
-        <v>-2.2889039419712902</v>
+        <v>-6.9469303891752796</v>
       </c>
       <c r="H121" s="12">
-        <v>18.9662833166926</v>
+        <v>16.810941165149298</v>
       </c>
       <c r="I121" s="12">
-        <v>3.1651334114635201</v>
+        <v>1.7078946819154801</v>
       </c>
       <c r="K121" s="1"/>
     </row>
@@ -11335,25 +11363,25 @@
         <v>9</v>
       </c>
       <c r="C122" s="12">
-        <v>16.1802925760467</v>
+        <v>15.728218306934499</v>
       </c>
       <c r="D122" s="12">
-        <v>11.974544160933901</v>
+        <v>9.4359568304784194</v>
       </c>
       <c r="E122" s="12">
-        <v>-5.6614115014834798</v>
+        <v>-6.9454109298056403</v>
       </c>
       <c r="F122" s="12">
         <v>16.714827162760098</v>
       </c>
       <c r="G122" s="12">
-        <v>9.49079036829648</v>
+        <v>5.1119977942698096</v>
       </c>
       <c r="H122" s="12">
-        <v>6.3896810174956</v>
+        <v>4.0541294601090101</v>
       </c>
       <c r="I122" s="12">
-        <v>10.194478189113401</v>
+        <v>8.7082869611133003</v>
       </c>
       <c r="K122" s="1"/>
     </row>
@@ -11362,25 +11390,25 @@
         <v>10</v>
       </c>
       <c r="C123" s="12">
-        <v>0.57655280366217798</v>
+        <v>0.21207556516316101</v>
       </c>
       <c r="D123" s="12">
-        <v>-8.1868357050396398E-2</v>
+        <v>-2.3626438850909302</v>
       </c>
       <c r="E123" s="12">
-        <v>-14.657993796920801</v>
+        <v>-15.7613242959128</v>
       </c>
       <c r="F123" s="12">
         <v>15.343608282550001</v>
       </c>
       <c r="G123" s="12">
-        <v>-1.5204325546550701</v>
+        <v>-6.0251161123711103</v>
       </c>
       <c r="H123" s="12">
-        <v>4.1775210369299902</v>
+        <v>2.0318606738557201</v>
       </c>
       <c r="I123" s="12">
-        <v>-1.3444392397132101</v>
+        <v>-2.6854342553846902</v>
       </c>
       <c r="K123" s="1"/>
     </row>
@@ -11389,25 +11417,25 @@
         <v>11</v>
       </c>
       <c r="C124" s="12">
-        <v>2.1201623244404302</v>
+        <v>1.7946106529942201</v>
       </c>
       <c r="D124" s="12">
-        <v>-3.7559979561316599</v>
+        <v>-6.1703330651894301</v>
       </c>
       <c r="E124" s="12">
-        <v>-22.411268647167599</v>
+        <v>-23.549430295908</v>
       </c>
       <c r="F124" s="12">
         <v>18.123377294566499</v>
       </c>
       <c r="G124" s="12">
-        <v>-1.3542187162241599</v>
+        <v>-5.7382181027617403</v>
       </c>
       <c r="H124" s="12">
-        <v>5.6151789259897704</v>
+        <v>3.3148109138884299</v>
       </c>
       <c r="I124" s="12">
-        <v>-2.8613489928644902</v>
+        <v>-4.2438261556003098</v>
       </c>
       <c r="K124" s="1"/>
     </row>
@@ -11415,13 +11443,27 @@
       <c r="B125" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="C125" s="16"/>
-      <c r="D125" s="16"/>
-      <c r="E125" s="16"/>
-      <c r="F125" s="16"/>
-      <c r="G125" s="16"/>
-      <c r="H125" s="16"/>
-      <c r="I125" s="16"/>
+      <c r="C125" s="16">
+        <v>3.2872010205948099</v>
+      </c>
+      <c r="D125" s="16">
+        <v>0.87832652466968097</v>
+      </c>
+      <c r="E125" s="16">
+        <v>-10.6925314759555</v>
+      </c>
+      <c r="F125" s="16">
+        <v>14.880875911357499</v>
+      </c>
+      <c r="G125" s="16">
+        <v>-5.3465863171995496</v>
+      </c>
+      <c r="H125" s="16">
+        <v>2.55776769111888</v>
+      </c>
+      <c r="I125" s="16">
+        <v>0.54332105714072199</v>
+      </c>
       <c r="K125" s="1"/>
     </row>
     <row r="126" spans="2:11" ht="14.25" customHeight="1">

</xml_diff>

<commit_message>
auto: actualizar datos del INE 2026-10-26
</commit_message>
<xml_diff>
--- a/datos/indicadores_adelantados/energia/indice_consumo_energia_electrica_2017_2026.xlsx
+++ b/datos/indicadores_adelantados/energia/indice_consumo_energia_electrica_2017_2026.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\1. Página Web\2026 - 09. Septiembre\Servicios Básicos 07-2026\PAGINA WEB JULIO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\1. Página Web\2026 - 10 Octubre\Servicios Básicos 08-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11130"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15525" windowHeight="8040"/>
   </bookViews>
   <sheets>
     <sheet name="Índice" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="37">
   <si>
     <t>DOMÉSTICO</t>
   </si>
@@ -269,9 +269,6 @@
   </si>
   <si>
     <t>BOLIVIA: VARIACIÓN A 12 MESES DEL ÍNDICE DE VOLUMEN DE CONSUMO DE ENERGÍA ELÉCTRICA POR CATEGORÍA, 2018 - 2026</t>
-  </si>
-  <si>
-    <t>2026(p)</t>
   </si>
 </sst>
 </file>
@@ -1099,7 +1096,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="B1:W171"/>
+  <dimension ref="B1:W172"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.28515625" customWidth="1"/>
@@ -4533,25 +4530,25 @@
         <v>33</v>
       </c>
       <c r="C132" s="10">
-        <v>122.88877997023801</v>
+        <v>123.29765466720301</v>
       </c>
       <c r="D132" s="10">
-        <v>122.15094187733</v>
+        <v>125.19887678859</v>
       </c>
       <c r="E132" s="10">
-        <v>117.300517005877</v>
+        <v>120.256171789652</v>
       </c>
       <c r="F132" s="10">
-        <v>183.181873589394</v>
+        <v>185.130973252415</v>
       </c>
       <c r="G132" s="10">
-        <v>112.019864578366</v>
+        <v>117.825071558034</v>
       </c>
       <c r="H132" s="10">
-        <v>158.93205939791699</v>
+        <v>164.77416037817201</v>
       </c>
       <c r="I132" s="10">
-        <v>125.259801752</v>
+        <v>127.475070766966</v>
       </c>
     </row>
     <row r="133" spans="2:9">
@@ -4559,25 +4556,25 @@
         <v>6</v>
       </c>
       <c r="C133" s="12">
-        <v>133.13831198384199</v>
+        <v>133.81745310174699</v>
       </c>
       <c r="D133" s="12">
-        <v>127.271341585988</v>
+        <v>130.315067629449</v>
       </c>
       <c r="E133" s="12">
-        <v>115.834787463176</v>
+        <v>117.55876343064899</v>
       </c>
       <c r="F133" s="12">
         <v>171.086962259134</v>
       </c>
       <c r="G133" s="12">
-        <v>110.277862718798</v>
+        <v>115.76923599584499</v>
       </c>
       <c r="H133" s="12">
-        <v>149.66492868690699</v>
+        <v>152.85179416885401</v>
       </c>
       <c r="I133" s="12">
-        <v>129.39004974020199</v>
+        <v>131.275379933279</v>
       </c>
     </row>
     <row r="134" spans="2:9">
@@ -4585,25 +4582,25 @@
         <v>7</v>
       </c>
       <c r="C134" s="12">
-        <v>129.776778725421</v>
+        <v>130.45201169262</v>
       </c>
       <c r="D134" s="12">
-        <v>127.81869034118699</v>
+        <v>130.87266117091599</v>
       </c>
       <c r="E134" s="12">
-        <v>115.47076275844501</v>
+        <v>117.192635509624</v>
       </c>
       <c r="F134" s="12">
         <v>173.441249375523</v>
       </c>
       <c r="G134" s="12">
-        <v>95.569212828195006</v>
+        <v>100.571432663838</v>
       </c>
       <c r="H134" s="12">
-        <v>150.55281705313101</v>
+        <v>153.57623840542101</v>
       </c>
       <c r="I134" s="12">
-        <v>127.411331799864</v>
+        <v>129.26183797899</v>
       </c>
     </row>
     <row r="135" spans="2:9">
@@ -4611,25 +4608,25 @@
         <v>8</v>
       </c>
       <c r="C135" s="12">
-        <v>128.221799364887</v>
+        <v>128.84501269150601</v>
       </c>
       <c r="D135" s="12">
-        <v>127.69149669452</v>
+        <v>130.74387424263199</v>
       </c>
       <c r="E135" s="12">
-        <v>122.65883552751799</v>
+        <v>124.35357664608399</v>
       </c>
       <c r="F135" s="12">
         <v>168.02622962471301</v>
       </c>
       <c r="G135" s="12">
-        <v>107.467631901583</v>
+        <v>112.84721877291901</v>
       </c>
       <c r="H135" s="12">
-        <v>165.62477124564001</v>
+        <v>168.68080390186901</v>
       </c>
       <c r="I135" s="12">
-        <v>129.06711750235101</v>
+        <v>130.91635057244599</v>
       </c>
     </row>
     <row r="136" spans="2:9">
@@ -4637,25 +4634,25 @@
         <v>9</v>
       </c>
       <c r="C136" s="12">
-        <v>129.56092972302201</v>
+        <v>130.06703932590801</v>
       </c>
       <c r="D136" s="12">
-        <v>132.03452004017501</v>
+        <v>135.09732653873701</v>
       </c>
       <c r="E136" s="12">
-        <v>129.16564495852299</v>
+        <v>130.94791723485801</v>
       </c>
       <c r="F136" s="12">
         <v>191.016110680964</v>
       </c>
       <c r="G136" s="12">
-        <v>126.486472253092</v>
+        <v>131.75569020193799</v>
       </c>
       <c r="H136" s="12">
-        <v>158.12208171700701</v>
+        <v>161.671217884187</v>
       </c>
       <c r="I136" s="12">
-        <v>134.06453787532701</v>
+        <v>135.89738379486101</v>
       </c>
     </row>
     <row r="137" spans="2:9">
@@ -4663,25 +4660,25 @@
         <v>10</v>
       </c>
       <c r="C137" s="12">
-        <v>116.153352096899</v>
+        <v>116.575808699818</v>
       </c>
       <c r="D137" s="12">
-        <v>119.03259659536199</v>
+        <v>121.813157685467</v>
       </c>
       <c r="E137" s="12">
-        <v>117.603891163109</v>
+        <v>119.14422829253201</v>
       </c>
       <c r="F137" s="12">
         <v>187.73390481546099</v>
       </c>
       <c r="G137" s="12">
-        <v>115.090461712289</v>
+        <v>120.60731993097301</v>
       </c>
       <c r="H137" s="12">
-        <v>157.631959331639</v>
+        <v>160.950357651329</v>
       </c>
       <c r="I137" s="12">
-        <v>122.18709595877699</v>
+        <v>123.870955926082</v>
       </c>
     </row>
     <row r="138" spans="2:9">
@@ -4689,109 +4686,126 @@
         <v>11</v>
       </c>
       <c r="C138" s="12">
-        <v>110.759533101789</v>
+        <v>111.113755696665</v>
       </c>
       <c r="D138" s="12">
-        <v>109.73253555183901</v>
+        <v>112.556068042611</v>
       </c>
       <c r="E138" s="12">
-        <v>98.978303686929806</v>
+        <v>100.45184809281</v>
       </c>
       <c r="F138" s="12">
         <v>194.36412997321901</v>
       </c>
       <c r="G138" s="12">
-        <v>113.32452378587899</v>
+        <v>118.59510782065399</v>
       </c>
       <c r="H138" s="12">
-        <v>162.77449867730201</v>
+        <v>166.40321059145401</v>
       </c>
       <c r="I138" s="12">
-        <v>114.46685207767401</v>
+        <v>116.119617814043</v>
       </c>
     </row>
     <row r="139" spans="2:9">
-      <c r="B139" s="33" t="s">
+      <c r="B139" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C139" s="16">
-        <v>112.61075479580801</v>
-      </c>
-      <c r="D139" s="16">
-        <v>111.47541233224</v>
-      </c>
-      <c r="E139" s="16">
-        <v>121.39139348344099</v>
-      </c>
-      <c r="F139" s="16">
+      <c r="C139" s="12">
+        <v>112.970109253217</v>
+      </c>
+      <c r="D139" s="12">
+        <v>114.309683134431</v>
+      </c>
+      <c r="E139" s="12">
+        <v>122.86642670821399</v>
+      </c>
+      <c r="F139" s="12">
         <v>196.60452839674201</v>
       </c>
-      <c r="G139" s="16">
-        <v>115.922886848723</v>
-      </c>
-      <c r="H139" s="16">
-        <v>168.15335907379099</v>
-      </c>
-      <c r="I139" s="16">
-        <v>120.23162730980199</v>
-      </c>
-    </row>
-    <row r="140" spans="2:9" ht="14.25" customHeight="1">
-      <c r="B140" s="29" t="s">
+      <c r="G139" s="12">
+        <v>121.37750835662899</v>
+      </c>
+      <c r="H139" s="12">
+        <v>171.982112440419</v>
+      </c>
+      <c r="I139" s="12">
+        <v>121.907955820864</v>
+      </c>
+    </row>
+    <row r="140" spans="2:9">
+      <c r="B140" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="C140" s="16">
+        <v>122.540046876142</v>
+      </c>
+      <c r="D140" s="16">
+        <v>125.88317586447999</v>
+      </c>
+      <c r="E140" s="16">
+        <v>129.533978402445</v>
+      </c>
+      <c r="F140" s="16">
+        <v>198.77467089356301</v>
+      </c>
+      <c r="G140" s="16">
+        <v>121.077058721477</v>
+      </c>
+      <c r="H140" s="16">
+        <v>182.07754798184001</v>
+      </c>
+      <c r="I140" s="16">
+        <v>130.55108429516201</v>
+      </c>
+    </row>
+    <row r="141" spans="2:9" ht="14.25" customHeight="1">
+      <c r="B141" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C140" s="30"/>
-      <c r="D140" s="30"/>
-      <c r="E140" s="30"/>
-      <c r="F140" s="30"/>
-      <c r="G140" s="30"/>
-      <c r="H140" s="30"/>
-      <c r="I140" s="30"/>
-    </row>
-    <row r="141" spans="2:9" ht="34.5" customHeight="1">
-      <c r="B141" s="35" t="s">
+      <c r="C141" s="30"/>
+      <c r="D141" s="30"/>
+      <c r="E141" s="30"/>
+      <c r="F141" s="30"/>
+      <c r="G141" s="30"/>
+      <c r="H141" s="30"/>
+      <c r="I141" s="30"/>
+    </row>
+    <row r="142" spans="2:9" ht="34.5" customHeight="1">
+      <c r="B142" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="C141" s="35"/>
-      <c r="D141" s="35"/>
-      <c r="E141" s="35"/>
-      <c r="F141" s="35"/>
-      <c r="G141" s="35"/>
-      <c r="H141" s="35"/>
-      <c r="I141" s="35"/>
-    </row>
-    <row r="142" spans="2:9">
-      <c r="B142" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="C142" s="32"/>
-      <c r="D142" s="32"/>
-      <c r="E142" s="32"/>
-      <c r="F142" s="32"/>
-      <c r="G142" s="32"/>
-      <c r="H142" s="32"/>
-      <c r="I142" s="32"/>
+      <c r="C142" s="35"/>
+      <c r="D142" s="35"/>
+      <c r="E142" s="35"/>
+      <c r="F142" s="35"/>
+      <c r="G142" s="35"/>
+      <c r="H142" s="35"/>
+      <c r="I142" s="35"/>
     </row>
     <row r="143" spans="2:9">
       <c r="B143" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C143" s="32"/>
+      <c r="D143" s="32"/>
+      <c r="E143" s="32"/>
+      <c r="F143" s="32"/>
+      <c r="G143" s="32"/>
+      <c r="H143" s="32"/>
+      <c r="I143" s="32"/>
+    </row>
+    <row r="144" spans="2:9">
+      <c r="B144" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="C143" s="30"/>
-      <c r="D143" s="30"/>
-      <c r="E143" s="30"/>
-      <c r="F143" s="30"/>
-      <c r="G143" s="30"/>
-      <c r="H143" s="30"/>
-      <c r="I143" s="30"/>
-    </row>
-    <row r="145" spans="3:9">
-      <c r="C145" s="17"/>
-      <c r="D145" s="17"/>
-      <c r="E145" s="17"/>
-      <c r="F145" s="17"/>
-      <c r="G145" s="17"/>
-      <c r="H145" s="17"/>
-      <c r="I145" s="17"/>
+      <c r="C144" s="30"/>
+      <c r="D144" s="30"/>
+      <c r="E144" s="30"/>
+      <c r="F144" s="30"/>
+      <c r="G144" s="30"/>
+      <c r="H144" s="30"/>
+      <c r="I144" s="30"/>
     </row>
     <row r="146" spans="3:9">
       <c r="C146" s="17"/>
@@ -4947,13 +4961,13 @@
       <c r="I162" s="17"/>
     </row>
     <row r="163" spans="3:9">
-      <c r="C163" s="18"/>
-      <c r="D163" s="18"/>
-      <c r="E163" s="18"/>
-      <c r="F163" s="18"/>
-      <c r="G163" s="18"/>
-      <c r="H163" s="18"/>
-      <c r="I163" s="18"/>
+      <c r="C163" s="17"/>
+      <c r="D163" s="17"/>
+      <c r="E163" s="17"/>
+      <c r="F163" s="17"/>
+      <c r="G163" s="17"/>
+      <c r="H163" s="17"/>
+      <c r="I163" s="17"/>
     </row>
     <row r="164" spans="3:9">
       <c r="C164" s="18"/>
@@ -5027,10 +5041,19 @@
       <c r="H171" s="18"/>
       <c r="I171" s="18"/>
     </row>
+    <row r="172" spans="3:9">
+      <c r="C172" s="18"/>
+      <c r="D172" s="18"/>
+      <c r="E172" s="18"/>
+      <c r="F172" s="18"/>
+      <c r="G172" s="18"/>
+      <c r="H172" s="18"/>
+      <c r="I172" s="18"/>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B141:I141"/>
+    <mergeCell ref="B142:I142"/>
     <mergeCell ref="B3:G3"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
@@ -5043,7 +5066,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Hoja3"/>
-  <dimension ref="B1:K151"/>
+  <dimension ref="B1:K152"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.28515625" customWidth="1"/>
@@ -7905,25 +7928,25 @@
         <v>33</v>
       </c>
       <c r="C118" s="10">
-        <v>3.1992428821396399</v>
+        <v>4.0286765918569802</v>
       </c>
       <c r="D118" s="10">
-        <v>-0.341613721558645</v>
+        <v>2.5002200663502201</v>
       </c>
       <c r="E118" s="10">
-        <v>-9.7537102968022502</v>
+        <v>-7.9189281386993304</v>
       </c>
       <c r="F118" s="10">
-        <v>16.067307000241101</v>
+        <v>17.1309300627676</v>
       </c>
       <c r="G118" s="10">
-        <v>-4.0999840497543003</v>
+        <v>0.18305974645325301</v>
       </c>
       <c r="H118" s="10">
-        <v>3.2118276840339899</v>
+        <v>4.9310125038884998</v>
       </c>
       <c r="I118" s="10">
-        <v>0.45838146946684299</v>
+        <v>2.3165824393207401</v>
       </c>
       <c r="J118" s="1"/>
       <c r="K118" s="1"/>
@@ -7933,25 +7956,25 @@
         <v>6</v>
       </c>
       <c r="C119" s="12">
-        <v>6.7555223386386798</v>
+        <v>7.3000843336288801</v>
       </c>
       <c r="D119" s="12">
-        <v>-2.0190457723200401</v>
+        <v>0.32419331379016603</v>
       </c>
       <c r="E119" s="12">
-        <v>-10.313128159798</v>
+        <v>-8.9783131613286002</v>
       </c>
       <c r="F119" s="12">
         <v>-11.3296548989108</v>
       </c>
       <c r="G119" s="12">
-        <v>0.17102600070926199</v>
+        <v>5.1591213604943702</v>
       </c>
       <c r="H119" s="12">
-        <v>-12.696527175261201</v>
+        <v>-10.837545071435599</v>
       </c>
       <c r="I119" s="12">
-        <v>-0.99663846481280505</v>
+        <v>0.44593016463887503</v>
       </c>
       <c r="J119" s="1"/>
       <c r="K119" s="1"/>
@@ -7961,25 +7984,25 @@
         <v>7</v>
       </c>
       <c r="C120" s="12">
-        <v>-2.5248429308832301</v>
+        <v>-2.5149495309616499</v>
       </c>
       <c r="D120" s="12">
-        <v>0.43006441857098598</v>
+        <v>0.42788109741207497</v>
       </c>
       <c r="E120" s="12">
-        <v>-0.31426198701000102</v>
+        <v>-0.31144247382378598</v>
       </c>
       <c r="F120" s="12">
         <v>1.37607628617773</v>
       </c>
       <c r="G120" s="12">
-        <v>-13.337808267203201</v>
+        <v>-13.127670059558801</v>
       </c>
       <c r="H120" s="12">
-        <v>0.59325078628282801</v>
+        <v>0.47395206612104201</v>
       </c>
       <c r="I120" s="12">
-        <v>-1.5292659244748299</v>
+        <v>-1.5338306050327</v>
       </c>
       <c r="J120" s="1"/>
       <c r="K120" s="1"/>
@@ -7989,25 +8012,25 @@
         <v>8</v>
       </c>
       <c r="C121" s="12">
-        <v>-1.19819537501703</v>
+        <v>-1.23186985027123</v>
       </c>
       <c r="D121" s="12">
-        <v>-9.9510991959073106E-2</v>
+        <v>-9.8406288319763405E-2</v>
       </c>
       <c r="E121" s="12">
-        <v>6.2250154042107004</v>
+        <v>6.11040199353834</v>
       </c>
       <c r="F121" s="12">
         <v>-3.12210605626229</v>
       </c>
       <c r="G121" s="12">
-        <v>12.450054490642</v>
+        <v>12.2060368276878</v>
       </c>
       <c r="H121" s="12">
-        <v>10.011074178167</v>
+        <v>9.8352229832417297</v>
       </c>
       <c r="I121" s="12">
-        <v>1.2995592143152199</v>
+        <v>1.27996988076684</v>
       </c>
       <c r="J121" s="1"/>
       <c r="K121" s="1"/>
@@ -8017,25 +8040,25 @@
         <v>9</v>
       </c>
       <c r="C122" s="12">
-        <v>1.04438587258016</v>
+        <v>0.94844698205578404</v>
       </c>
       <c r="D122" s="12">
-        <v>3.4011844626155501</v>
+        <v>3.3297562285986801</v>
       </c>
       <c r="E122" s="12">
-        <v>5.3048028729613099</v>
+        <v>5.3028957965092403</v>
       </c>
       <c r="F122" s="12">
         <v>13.682316807083801</v>
       </c>
       <c r="G122" s="12">
-        <v>17.6972731370189</v>
+        <v>16.755815193875701</v>
       </c>
       <c r="H122" s="12">
-        <v>-4.5299320096910396</v>
+        <v>-4.1555327313707</v>
       </c>
       <c r="I122" s="12">
-        <v>3.8719547392734399</v>
+        <v>3.80474493876015</v>
       </c>
       <c r="J122" s="1"/>
       <c r="K122" s="1"/>
@@ -8045,25 +8068,25 @@
         <v>10</v>
       </c>
       <c r="C123" s="12">
-        <v>-10.3484728419173</v>
+        <v>-10.372520737006401</v>
       </c>
       <c r="D123" s="12">
-        <v>-9.8473667650375099</v>
+        <v>-9.8330360737828997</v>
       </c>
       <c r="E123" s="12">
-        <v>-8.9511059996845095</v>
+        <v>-9.0140333588935899</v>
       </c>
       <c r="F123" s="12">
         <v>-1.7182874542895901</v>
       </c>
       <c r="G123" s="12">
-        <v>-9.0096674670474002</v>
+        <v>-8.4613956739772007</v>
       </c>
       <c r="H123" s="12">
-        <v>-0.30996454135048301</v>
+        <v>-0.44588037517879803</v>
       </c>
       <c r="I123" s="12">
-        <v>-8.8594956614067701</v>
+        <v>-8.8496389944734997</v>
       </c>
       <c r="J123" s="1"/>
       <c r="K123" s="1"/>
@@ -8073,121 +8096,140 @@
         <v>11</v>
       </c>
       <c r="C124" s="12">
-        <v>-4.6437049794399696</v>
+        <v>-4.6854086315777401</v>
       </c>
       <c r="D124" s="12">
-        <v>-7.81303719277635</v>
+        <v>-7.5994168600068397</v>
       </c>
       <c r="E124" s="12">
-        <v>-15.837560553457299</v>
+        <v>-15.6888675747067</v>
       </c>
       <c r="F124" s="12">
         <v>3.5317142975718201</v>
       </c>
       <c r="G124" s="12">
-        <v>-1.53439120856474</v>
+        <v>-1.66839965556889</v>
       </c>
       <c r="H124" s="12">
-        <v>3.26237101122608</v>
+        <v>3.3879098000750201</v>
       </c>
       <c r="I124" s="12">
-        <v>-6.3183790567443499</v>
+        <v>-6.2575912602661701</v>
       </c>
       <c r="J124" s="1"/>
       <c r="K124" s="1"/>
     </row>
     <row r="125" spans="2:11">
-      <c r="B125" s="33" t="s">
+      <c r="B125" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C125" s="16">
-        <v>1.67138813443486</v>
-      </c>
-      <c r="D125" s="16">
-        <v>1.58829536894929</v>
-      </c>
-      <c r="E125" s="16">
-        <v>22.644447279481099</v>
-      </c>
-      <c r="F125" s="16">
+      <c r="C125" s="12">
+        <v>1.67067843662843</v>
+      </c>
+      <c r="D125" s="12">
+        <v>1.55799249415567</v>
+      </c>
+      <c r="E125" s="12">
+        <v>22.3137543419755</v>
+      </c>
+      <c r="F125" s="12">
         <v>1.1526810136374599</v>
       </c>
-      <c r="G125" s="16">
-        <v>2.2928515170759698</v>
-      </c>
-      <c r="H125" s="16">
-        <v>3.3044859238994699</v>
-      </c>
-      <c r="I125" s="16">
-        <v>5.0361961803725697</v>
+      <c r="G125" s="12">
+        <v>2.3461343280558999</v>
+      </c>
+      <c r="H125" s="12">
+        <v>3.3526407508215099</v>
+      </c>
+      <c r="I125" s="12">
+        <v>4.9848062849210599</v>
       </c>
       <c r="J125" s="1"/>
       <c r="K125" s="1"/>
     </row>
-    <row r="126" spans="2:11" ht="14.25" customHeight="1">
-      <c r="B126" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="C126" s="30"/>
-      <c r="D126" s="30"/>
-      <c r="E126" s="30"/>
-      <c r="F126" s="30"/>
-      <c r="G126" s="30"/>
-      <c r="H126" s="30"/>
-      <c r="I126" s="30"/>
+    <row r="126" spans="2:11">
+      <c r="B126" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="C126" s="16">
+        <v>8.47121215176894</v>
+      </c>
+      <c r="D126" s="16">
+        <v>10.124682715144999</v>
+      </c>
+      <c r="E126" s="16">
+        <v>5.4266668876636697</v>
+      </c>
+      <c r="F126" s="16">
+        <v>1.1038110436813799</v>
+      </c>
+      <c r="G126" s="16">
+        <v>-0.24753320382008301</v>
+      </c>
+      <c r="H126" s="16">
+        <v>5.87004973841014</v>
+      </c>
+      <c r="I126" s="16">
+        <v>7.0898805710426496</v>
+      </c>
       <c r="J126" s="1"/>
       <c r="K126" s="1"/>
     </row>
-    <row r="127" spans="2:11" ht="34.5" customHeight="1">
-      <c r="B127" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="C127" s="35"/>
-      <c r="D127" s="35"/>
-      <c r="E127" s="35"/>
-      <c r="F127" s="35"/>
-      <c r="G127" s="35"/>
-      <c r="H127" s="35"/>
-      <c r="I127" s="35"/>
+    <row r="127" spans="2:11" ht="14.25" customHeight="1">
+      <c r="B127" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="C127" s="30"/>
+      <c r="D127" s="30"/>
+      <c r="E127" s="30"/>
+      <c r="F127" s="30"/>
+      <c r="G127" s="30"/>
+      <c r="H127" s="30"/>
+      <c r="I127" s="30"/>
       <c r="J127" s="1"/>
       <c r="K127" s="1"/>
     </row>
-    <row r="128" spans="2:11">
-      <c r="B128" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="C128" s="32"/>
-      <c r="D128" s="32"/>
-      <c r="E128" s="32"/>
-      <c r="F128" s="32"/>
-      <c r="G128" s="32"/>
-      <c r="H128" s="32"/>
-      <c r="I128" s="32"/>
+    <row r="128" spans="2:11" ht="34.5" customHeight="1">
+      <c r="B128" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="C128" s="35"/>
+      <c r="D128" s="35"/>
+      <c r="E128" s="35"/>
+      <c r="F128" s="35"/>
+      <c r="G128" s="35"/>
+      <c r="H128" s="35"/>
+      <c r="I128" s="35"/>
       <c r="J128" s="1"/>
       <c r="K128" s="1"/>
     </row>
     <row r="129" spans="2:11">
       <c r="B129" s="31" t="s">
-        <v>29</v>
-      </c>
-      <c r="C129" s="30"/>
-      <c r="D129" s="30"/>
-      <c r="E129" s="30"/>
-      <c r="F129" s="30"/>
-      <c r="G129" s="30"/>
-      <c r="H129" s="30"/>
-      <c r="I129" s="30"/>
+        <v>24</v>
+      </c>
+      <c r="C129" s="32"/>
+      <c r="D129" s="32"/>
+      <c r="E129" s="32"/>
+      <c r="F129" s="32"/>
+      <c r="G129" s="32"/>
+      <c r="H129" s="32"/>
+      <c r="I129" s="32"/>
       <c r="J129" s="1"/>
       <c r="K129" s="1"/>
     </row>
     <row r="130" spans="2:11">
-      <c r="C130" s="19"/>
-      <c r="D130" s="19"/>
-      <c r="E130" s="19"/>
-      <c r="F130" s="19"/>
-      <c r="G130" s="19"/>
-      <c r="H130" s="19"/>
-      <c r="I130" s="19"/>
+      <c r="B130" s="31" t="s">
+        <v>29</v>
+      </c>
+      <c r="C130" s="30"/>
+      <c r="D130" s="30"/>
+      <c r="E130" s="30"/>
+      <c r="F130" s="30"/>
+      <c r="G130" s="30"/>
+      <c r="H130" s="30"/>
+      <c r="I130" s="30"/>
+      <c r="J130" s="1"/>
+      <c r="K130" s="1"/>
     </row>
     <row r="131" spans="2:11">
       <c r="C131" s="19"/>
@@ -8226,13 +8268,13 @@
       <c r="I134" s="19"/>
     </row>
     <row r="135" spans="2:11">
-      <c r="C135" s="17"/>
-      <c r="D135" s="17"/>
-      <c r="E135" s="17"/>
-      <c r="F135" s="17"/>
-      <c r="G135" s="17"/>
-      <c r="H135" s="17"/>
-      <c r="I135" s="17"/>
+      <c r="C135" s="19"/>
+      <c r="D135" s="19"/>
+      <c r="E135" s="19"/>
+      <c r="F135" s="19"/>
+      <c r="G135" s="19"/>
+      <c r="H135" s="19"/>
+      <c r="I135" s="19"/>
     </row>
     <row r="136" spans="2:11">
       <c r="C136" s="17"/>
@@ -8378,10 +8420,19 @@
       <c r="H151" s="17"/>
       <c r="I151" s="17"/>
     </row>
+    <row r="152" spans="3:9">
+      <c r="C152" s="17"/>
+      <c r="D152" s="17"/>
+      <c r="E152" s="17"/>
+      <c r="F152" s="17"/>
+      <c r="G152" s="17"/>
+      <c r="H152" s="17"/>
+      <c r="I152" s="17"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B127:I127"/>
+    <mergeCell ref="B128:I128"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8393,7 +8444,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="B1:K160"/>
+  <dimension ref="B1:K161"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.28515625" customWidth="1"/>
@@ -11252,28 +11303,28 @@
     </row>
     <row r="118" spans="2:11">
       <c r="B118" s="9" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C118" s="10">
-        <v>3.1992428821396399</v>
+        <v>4.0286765918569802</v>
       </c>
       <c r="D118" s="10">
-        <v>-0.341613721558645</v>
+        <v>2.5002200663502201</v>
       </c>
       <c r="E118" s="10">
-        <v>-9.7537102968022502</v>
+        <v>-7.9189281386993304</v>
       </c>
       <c r="F118" s="10">
-        <v>16.067307000241101</v>
+        <v>17.1309300627676</v>
       </c>
       <c r="G118" s="10">
-        <v>-4.0999840497543003</v>
+        <v>0.18305974645325301</v>
       </c>
       <c r="H118" s="10">
-        <v>3.2118276840339899</v>
+        <v>4.9310125038884998</v>
       </c>
       <c r="I118" s="10">
-        <v>0.45838146946684299</v>
+        <v>2.3165824393207401</v>
       </c>
       <c r="K118" s="1"/>
     </row>
@@ -11282,25 +11333,25 @@
         <v>6</v>
       </c>
       <c r="C119" s="12">
-        <v>3.20221882389218</v>
+        <v>3.72865534857034</v>
       </c>
       <c r="D119" s="12">
-        <v>0.35187884253371499</v>
+        <v>2.7518191852456502</v>
       </c>
       <c r="E119" s="12">
-        <v>-3.98063621507624</v>
+        <v>-2.5515743658463301</v>
       </c>
       <c r="F119" s="12">
         <v>13.293318580951601</v>
       </c>
       <c r="G119" s="12">
-        <v>0.987327119532178</v>
+        <v>6.0160708382844801</v>
       </c>
       <c r="H119" s="12">
-        <v>-7.3592290027508902</v>
+        <v>-5.3865980203131096</v>
       </c>
       <c r="I119" s="12">
-        <v>1.43124165915374</v>
+        <v>2.9091867005634802</v>
       </c>
       <c r="K119" s="1"/>
     </row>
@@ -11309,25 +11360,25 @@
         <v>7</v>
       </c>
       <c r="C120" s="12">
-        <v>-1.5806376085685101</v>
+        <v>-1.0685583386863899</v>
       </c>
       <c r="D120" s="12">
-        <v>-2.7192067197782999</v>
+        <v>-0.39487759249986498</v>
       </c>
       <c r="E120" s="12">
-        <v>-7.7034325470668499</v>
+        <v>-6.3271279247704504</v>
       </c>
       <c r="F120" s="12">
         <v>14.561465258757099</v>
       </c>
       <c r="G120" s="12">
-        <v>-11.077136734808199</v>
+        <v>-6.4227956839202101</v>
       </c>
       <c r="H120" s="12">
-        <v>2.69959637236752</v>
+        <v>4.76202309158404</v>
       </c>
       <c r="I120" s="12">
-        <v>-2.2528765351399498</v>
+        <v>-0.83320959179789</v>
       </c>
       <c r="K120" s="1"/>
     </row>
@@ -11336,25 +11387,25 @@
         <v>8</v>
       </c>
       <c r="C121" s="12">
-        <v>0.96856155629183605</v>
+        <v>1.45931237591159</v>
       </c>
       <c r="D121" s="12">
-        <v>-1.58996733338195</v>
+        <v>0.76245692349070604</v>
       </c>
       <c r="E121" s="12">
-        <v>1.96449595597716</v>
+        <v>3.3733094604205101</v>
       </c>
       <c r="F121" s="12">
         <v>19.799265689296799</v>
       </c>
       <c r="G121" s="12">
-        <v>-6.9469303891752796</v>
+        <v>-2.2889039419712902</v>
       </c>
       <c r="H121" s="12">
-        <v>16.810941165149298</v>
+        <v>18.9662833166926</v>
       </c>
       <c r="I121" s="12">
-        <v>1.7078946819154801</v>
+        <v>3.1651334114635201</v>
       </c>
       <c r="K121" s="1"/>
     </row>
@@ -11363,25 +11414,25 @@
         <v>9</v>
       </c>
       <c r="C122" s="12">
-        <v>15.728218306934499</v>
+        <v>16.1802925760467</v>
       </c>
       <c r="D122" s="12">
-        <v>9.4359568304784194</v>
+        <v>11.974544160933901</v>
       </c>
       <c r="E122" s="12">
-        <v>-6.9454109298056403</v>
+        <v>-5.6614115014834798</v>
       </c>
       <c r="F122" s="12">
         <v>16.714827162760098</v>
       </c>
       <c r="G122" s="12">
-        <v>5.1119977942698096</v>
+        <v>9.49079036829648</v>
       </c>
       <c r="H122" s="12">
-        <v>4.0541294601090101</v>
+        <v>6.3896810174956</v>
       </c>
       <c r="I122" s="12">
-        <v>8.7082869611133003</v>
+        <v>10.194478189113401</v>
       </c>
       <c r="K122" s="1"/>
     </row>
@@ -11390,25 +11441,25 @@
         <v>10</v>
       </c>
       <c r="C123" s="12">
-        <v>0.21207556516316101</v>
+        <v>0.57655280366217798</v>
       </c>
       <c r="D123" s="12">
-        <v>-2.3626438850909302</v>
+        <v>-8.1868357050396398E-2</v>
       </c>
       <c r="E123" s="12">
-        <v>-15.7613242959128</v>
+        <v>-14.657993796920801</v>
       </c>
       <c r="F123" s="12">
         <v>15.343608282550001</v>
       </c>
       <c r="G123" s="12">
-        <v>-6.0251161123711103</v>
+        <v>-1.5204325546550701</v>
       </c>
       <c r="H123" s="12">
-        <v>2.0318606738557201</v>
+        <v>4.1797902970780498</v>
       </c>
       <c r="I123" s="12">
-        <v>-2.6854342553846902</v>
+        <v>-1.3443425451091899</v>
       </c>
       <c r="K123" s="1"/>
     </row>
@@ -11417,115 +11468,133 @@
         <v>11</v>
       </c>
       <c r="C124" s="12">
-        <v>1.7946106529942201</v>
+        <v>2.1201623244404302</v>
       </c>
       <c r="D124" s="12">
-        <v>-6.1703330651894301</v>
+        <v>-3.7559979561316599</v>
       </c>
       <c r="E124" s="12">
-        <v>-23.549430295908</v>
+        <v>-22.411268647167599</v>
       </c>
       <c r="F124" s="12">
         <v>18.123377294566499</v>
       </c>
       <c r="G124" s="12">
-        <v>-5.7382181027617403</v>
+        <v>-1.3542187162241599</v>
       </c>
       <c r="H124" s="12">
-        <v>3.3148109138884299</v>
+        <v>5.6179953089752201</v>
       </c>
       <c r="I124" s="12">
-        <v>-4.2438261556003098</v>
+        <v>-2.86122044658305</v>
       </c>
       <c r="K124" s="1"/>
     </row>
     <row r="125" spans="2:11">
-      <c r="B125" s="33" t="s">
+      <c r="B125" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C125" s="16">
-        <v>3.2872010205948099</v>
-      </c>
-      <c r="D125" s="16">
-        <v>0.87832652466968097</v>
-      </c>
-      <c r="E125" s="16">
-        <v>-10.6925314759555</v>
-      </c>
-      <c r="F125" s="16">
+      <c r="C125" s="12">
+        <v>3.6168028969643302</v>
+      </c>
+      <c r="D125" s="12">
+        <v>3.4431656175336398</v>
+      </c>
+      <c r="E125" s="12">
+        <v>-9.6073517155689991</v>
+      </c>
+      <c r="F125" s="12">
         <v>14.880875911357499</v>
       </c>
-      <c r="G125" s="16">
-        <v>-5.3465863171995496</v>
-      </c>
-      <c r="H125" s="16">
-        <v>2.55776769111888</v>
-      </c>
-      <c r="I125" s="16">
-        <v>0.54332105714072199</v>
+      <c r="G125" s="12">
+        <v>-0.89277602911833598</v>
+      </c>
+      <c r="H125" s="12">
+        <v>4.8929479128167603</v>
+      </c>
+      <c r="I125" s="12">
+        <v>1.94514551428282</v>
       </c>
       <c r="K125" s="1"/>
     </row>
-    <row r="126" spans="2:11" ht="14.25" customHeight="1">
-      <c r="B126" s="29" t="s">
+    <row r="126" spans="2:11">
+      <c r="B126" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="C126" s="16">
+        <v>6.9023613107201296</v>
+      </c>
+      <c r="D126" s="16">
+        <v>5.6312639641402704</v>
+      </c>
+      <c r="E126" s="16">
+        <v>-4.0045700279171896</v>
+      </c>
+      <c r="F126" s="16">
+        <v>24.490159706486399</v>
+      </c>
+      <c r="G126" s="16">
+        <v>-1.7352057412665001</v>
+      </c>
+      <c r="H126" s="16">
+        <v>2.0937038198495501</v>
+      </c>
+      <c r="I126" s="16">
+        <v>5.3739254579769904</v>
+      </c>
+      <c r="K126" s="1"/>
+    </row>
+    <row r="127" spans="2:11" ht="14.25" customHeight="1">
+      <c r="B127" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C126" s="30"/>
-      <c r="D126" s="30"/>
-      <c r="E126" s="30"/>
-      <c r="F126" s="30"/>
-      <c r="G126" s="30"/>
-      <c r="H126" s="30"/>
-      <c r="I126" s="30"/>
-      <c r="K126" s="1"/>
-    </row>
-    <row r="127" spans="2:11" ht="34.5" customHeight="1">
-      <c r="B127" s="35" t="s">
+      <c r="C127" s="30"/>
+      <c r="D127" s="30"/>
+      <c r="E127" s="30"/>
+      <c r="F127" s="30"/>
+      <c r="G127" s="30"/>
+      <c r="H127" s="30"/>
+      <c r="I127" s="30"/>
+      <c r="K127" s="1"/>
+    </row>
+    <row r="128" spans="2:11" ht="34.5" customHeight="1">
+      <c r="B128" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="C127" s="35"/>
-      <c r="D127" s="35"/>
-      <c r="E127" s="35"/>
-      <c r="F127" s="35"/>
-      <c r="G127" s="35"/>
-      <c r="H127" s="35"/>
-      <c r="I127" s="35"/>
-      <c r="K127" s="1"/>
-    </row>
-    <row r="128" spans="2:11">
-      <c r="B128" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="C128" s="32"/>
-      <c r="D128" s="32"/>
-      <c r="E128" s="32"/>
-      <c r="F128" s="32"/>
-      <c r="G128" s="32"/>
-      <c r="H128" s="32"/>
-      <c r="I128" s="32"/>
+      <c r="C128" s="35"/>
+      <c r="D128" s="35"/>
+      <c r="E128" s="35"/>
+      <c r="F128" s="35"/>
+      <c r="G128" s="35"/>
+      <c r="H128" s="35"/>
+      <c r="I128" s="35"/>
       <c r="K128" s="1"/>
     </row>
     <row r="129" spans="2:11">
       <c r="B129" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C129" s="32"/>
+      <c r="D129" s="32"/>
+      <c r="E129" s="32"/>
+      <c r="F129" s="32"/>
+      <c r="G129" s="32"/>
+      <c r="H129" s="32"/>
+      <c r="I129" s="32"/>
+      <c r="K129" s="1"/>
+    </row>
+    <row r="130" spans="2:11">
+      <c r="B130" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="C129" s="30"/>
-      <c r="D129" s="30"/>
-      <c r="E129" s="30"/>
-      <c r="F129" s="30"/>
-      <c r="G129" s="30"/>
-      <c r="H129" s="30"/>
-      <c r="I129" s="30"/>
-      <c r="K129" s="1"/>
-    </row>
-    <row r="134" spans="2:11">
-      <c r="C134" s="17"/>
-      <c r="D134" s="17"/>
-      <c r="E134" s="17"/>
-      <c r="F134" s="17"/>
-      <c r="G134" s="17"/>
-      <c r="H134" s="17"/>
-      <c r="I134" s="17"/>
+      <c r="C130" s="30"/>
+      <c r="D130" s="30"/>
+      <c r="E130" s="30"/>
+      <c r="F130" s="30"/>
+      <c r="G130" s="30"/>
+      <c r="H130" s="30"/>
+      <c r="I130" s="30"/>
+      <c r="K130" s="1"/>
     </row>
     <row r="135" spans="2:11">
       <c r="C135" s="17"/>
@@ -11635,14 +11704,14 @@
       <c r="H146" s="17"/>
       <c r="I146" s="17"/>
     </row>
-    <row r="149" spans="3:9">
-      <c r="C149" s="17"/>
-      <c r="D149" s="17"/>
-      <c r="E149" s="17"/>
-      <c r="F149" s="17"/>
-      <c r="G149" s="17"/>
-      <c r="H149" s="17"/>
-      <c r="I149" s="17"/>
+    <row r="147" spans="3:9">
+      <c r="C147" s="17"/>
+      <c r="D147" s="17"/>
+      <c r="E147" s="17"/>
+      <c r="F147" s="17"/>
+      <c r="G147" s="17"/>
+      <c r="H147" s="17"/>
+      <c r="I147" s="17"/>
     </row>
     <row r="150" spans="3:9">
       <c r="C150" s="17"/>
@@ -11743,14 +11812,23 @@
       <c r="H160" s="17"/>
       <c r="I160" s="17"/>
     </row>
+    <row r="161" spans="3:9">
+      <c r="C161" s="17"/>
+      <c r="D161" s="17"/>
+      <c r="E161" s="17"/>
+      <c r="F161" s="17"/>
+      <c r="G161" s="17"/>
+      <c r="H161" s="17"/>
+      <c r="I161" s="17"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B127:I127"/>
+    <mergeCell ref="B128:I128"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>